<commit_message>
feat: add some examples to import template
</commit_message>
<xml_diff>
--- a/template/public/template.xlsx
+++ b/template/public/template.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="119">
   <si>
     <t xml:space="preserve">site_code</t>
   </si>
@@ -125,6 +125,9 @@
     <t xml:space="preserve">pub_verbatim</t>
   </si>
   <si>
+    <t xml:space="preserve">occurrence_id</t>
+  </si>
+  <si>
     <t xml:space="preserve">gene</t>
   </si>
   <si>
@@ -143,9 +146,6 @@
     <t xml:space="preserve">sampling_effort</t>
   </si>
   <si>
-    <t xml:space="preserve">occurrence_id</t>
-  </si>
-  <si>
     <t xml:space="preserve">PIVKACAV</t>
   </si>
   <si>
@@ -212,6 +212,12 @@
     <t xml:space="preserve">MERAVIGL</t>
   </si>
   <si>
+    <t xml:space="preserve">45.688</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.7888</t>
+  </si>
+  <si>
     <t xml:space="preserve">ITA</t>
   </si>
   <si>
@@ -245,9 +251,6 @@
     <t xml:space="preserve">KT364292</t>
   </si>
   <si>
-    <t xml:space="preserve">NA</t>
-  </si>
-  <si>
     <t xml:space="preserve">JE7</t>
   </si>
   <si>
@@ -263,6 +266,12 @@
     <t xml:space="preserve">TREBICGR</t>
   </si>
   <si>
+    <t xml:space="preserve">45.685327</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.833536</t>
+  </si>
+  <si>
     <t xml:space="preserve">Douady, Christophe | Lefebure, Tristan | Malard, Florian|Mauri, E</t>
   </si>
   <si>
@@ -276,6 +285,99 @@
   </si>
   <si>
     <t xml:space="preserve">10.1016/j.jcz.2009.03.001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SIPANFON</t>
+  </si>
+  <si>
+    <t xml:space="preserve">42.1831</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.2659</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sipan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Douady,Christophe | Malard, Florian | Morvan, C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surber net</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proasellus lescherae, Stenasellus virei virei</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aquatic, Subsurface, Aquifer, Freshwater, Porous</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fountain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proasellus lescherae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proasellus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">true</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2010-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Several</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 specimens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GUADALQ1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38.0628</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-2.83025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coto Rìos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notenboom, J | Meijers, C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bou-Rouch pump</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Animalia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aquatic, Subsurface, Aquifer, Hyporheic zone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hyporheic zone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proasellus aff. Escolai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Henry, J P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 juveniles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Henry J.-P., Magniez G.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">. Isopodes aselloides stygobies d Espagne, III - Le genre Proasellus: B - Especes anophtalmes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Henry J.-P., Magniez G. 2003. Isopodes aselloides stygobies d Espagne, III - Le genre Proasellus: B - Especes anophtalmes. Beaufortia, 53(6), 129-158.</t>
   </si>
 </sst>
 </file>
@@ -286,7 +388,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -360,8 +462,14 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -392,6 +500,12 @@
         <bgColor rgb="FF969696"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FFCCFFCC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border diagonalUp="false" diagonalDown="false">
@@ -427,7 +541,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -529,10 +643,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -552,8 +662,20 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -590,7 +712,7 @@
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FFD9D9D9"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -633,7 +755,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AS1"/>
+  <dimension ref="A1:AT1"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="11.53"/>
@@ -647,7 +769,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="13.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="14.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="15.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="13.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="13.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="13.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="19" style="1" width="14.6"/>
@@ -658,9 +780,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="1" width="16.69"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="1" width="20.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="33" style="1" width="13.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="1" width="21.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="1" width="20.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="1" width="19.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="1" width="14.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="1" width="21.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="1" width="20.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="1" width="19.47"/>
   </cols>
   <sheetData>
     <row r="1" s="10" customFormat="true" ht="29.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -778,15 +901,18 @@
       <c r="AL1" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" s="13" t="s">
+      <c r="AM1" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" s="1"/>
+      <c r="AN1" s="13" t="s">
+        <v>39</v>
+      </c>
       <c r="AO1" s="1"/>
       <c r="AP1" s="1"/>
       <c r="AQ1" s="1"/>
       <c r="AR1" s="1"/>
       <c r="AS1" s="1"/>
+      <c r="AT1" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -804,22 +930,22 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AO7"/>
+  <dimension ref="A1:AO9"/>
   <sheetFormatPr defaultColWidth="16.96484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="35.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="23.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="23.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="28.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="1" width="42.69"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="28.65"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="19.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="22.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="19.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="1" width="22.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="1" width="24.2"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="1" width="34.49"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="0" width="25.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="1" width="25.04"/>
   </cols>
   <sheetData>
-    <row r="1" s="27" customFormat="true" ht="29.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" s="26" customFormat="true" ht="29.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
@@ -857,7 +983,7 @@
         <v>11</v>
       </c>
       <c r="M1" s="18" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="N1" s="17" t="s">
         <v>12</v>
@@ -925,291 +1051,435 @@
       <c r="AI1" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="AJ1" s="25" t="s">
-        <v>40</v>
+      <c r="AJ1" s="22" t="s">
+        <v>34</v>
       </c>
       <c r="AK1" s="22" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="AL1" s="22" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="AM1" s="22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="AN1" s="22" t="s">
-        <v>37</v>
-      </c>
-      <c r="AO1" s="26" t="s">
         <v>38</v>
       </c>
+      <c r="AO1" s="25" t="s">
+        <v>39</v>
+      </c>
     </row>
-    <row r="2" s="28" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="28" t="s">
+    <row r="2" s="27" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="C2" s="28" t="s">
+      <c r="C2" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="D2" s="28" t="s">
+      <c r="D2" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="28" t="n">
+      <c r="E2" s="27" t="n">
         <v>526</v>
       </c>
-      <c r="F2" s="28" t="s">
+      <c r="F2" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="G2" s="28" t="s">
+      <c r="G2" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="H2" s="29" t="n">
+      <c r="H2" s="28" t="n">
         <v>34023</v>
       </c>
-      <c r="I2" s="28" t="s">
+      <c r="I2" s="27" t="s">
         <v>47</v>
       </c>
-      <c r="J2" s="28" t="s">
+      <c r="J2" s="27" t="s">
         <v>48</v>
       </c>
-      <c r="K2" s="28" t="s">
+      <c r="K2" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="L2" s="28" t="s">
+      <c r="L2" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="N2" s="28" t="s">
+      <c r="N2" s="27" t="s">
         <v>51</v>
       </c>
-      <c r="O2" s="28" t="s">
+      <c r="O2" s="27" t="s">
         <v>52</v>
       </c>
-      <c r="Q2" s="28" t="s">
+      <c r="Q2" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="R2" s="28" t="s">
+      <c r="R2" s="27" t="s">
         <v>53</v>
       </c>
-      <c r="S2" s="28" t="s">
+      <c r="S2" s="27" t="s">
         <v>54</v>
       </c>
-      <c r="T2" s="28" t="s">
+      <c r="T2" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="U2" s="28" t="s">
+      <c r="U2" s="27" t="s">
         <v>56</v>
       </c>
-      <c r="X2" s="29" t="n">
+      <c r="X2" s="28" t="n">
         <v>34023</v>
       </c>
-      <c r="Y2" s="28" t="s">
+      <c r="Y2" s="27" t="s">
         <v>57</v>
       </c>
-      <c r="Z2" s="28" t="s">
+      <c r="Z2" s="27" t="s">
         <v>58</v>
       </c>
-      <c r="AA2" s="28" t="s">
+      <c r="AA2" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="AC2" s="28" t="s">
+      <c r="AC2" s="27" t="s">
         <v>60</v>
       </c>
-      <c r="AD2" s="30" t="s">
+      <c r="AD2" s="29" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="3" s="31" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="28" t="s">
+    <row r="3" s="27" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="27" t="s">
         <v>62</v>
       </c>
-      <c r="B3" s="28" t="n">
-        <v>45.688</v>
-      </c>
-      <c r="C3" s="28" t="n">
-        <v>13.7888</v>
-      </c>
-      <c r="E3" s="28" t="n">
+      <c r="B3" s="27" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3" s="27" t="s">
+        <v>64</v>
+      </c>
+      <c r="E3" s="27" t="n">
         <v>322</v>
       </c>
-      <c r="F3" s="28" t="s">
-        <v>63</v>
-      </c>
-      <c r="G3" s="28" t="s">
-        <v>64</v>
-      </c>
-      <c r="L3" s="28" t="s">
+      <c r="F3" s="27" t="s">
         <v>65</v>
       </c>
-      <c r="M3" s="28"/>
-      <c r="N3" s="28" t="s">
+      <c r="G3" s="27" t="s">
         <v>66</v>
       </c>
-      <c r="O3" s="28" t="s">
+      <c r="L3" s="27" t="s">
+        <v>67</v>
+      </c>
+      <c r="N3" s="27" t="s">
+        <v>68</v>
+      </c>
+      <c r="O3" s="27" t="s">
         <v>52</v>
       </c>
-      <c r="Q3" s="28" t="s">
+      <c r="Q3" s="27" t="s">
+        <v>67</v>
+      </c>
+      <c r="R3" s="27" t="s">
+        <v>69</v>
+      </c>
+      <c r="S3" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="T3" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="X3" s="28" t="n">
+        <v>42993</v>
+      </c>
+      <c r="Y3" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="AD3" s="27" t="s">
+        <v>71</v>
+      </c>
+      <c r="AJ3" s="27" t="s">
+        <v>72</v>
+      </c>
+      <c r="AK3" s="27" t="s">
+        <v>73</v>
+      </c>
+      <c r="AL3" s="27" t="s">
+        <v>74</v>
+      </c>
+      <c r="AM3" s="27" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" s="27" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="AJ4" s="27" t="s">
+        <v>72</v>
+      </c>
+      <c r="AK4" s="27" t="s">
+        <v>73</v>
+      </c>
+      <c r="AL4" s="27" t="s">
+        <v>76</v>
+      </c>
+      <c r="AM4" s="27" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="5" s="27" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="AJ5" s="27" t="s">
+        <v>72</v>
+      </c>
+      <c r="AK5" s="27" t="s">
+        <v>73</v>
+      </c>
+      <c r="AL5" s="27" t="s">
+        <v>78</v>
+      </c>
+      <c r="AM5" s="27" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="6" s="27" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="27" t="s">
+        <v>80</v>
+      </c>
+      <c r="B6" s="27" t="s">
+        <v>81</v>
+      </c>
+      <c r="C6" s="27" t="s">
+        <v>82</v>
+      </c>
+      <c r="D6" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" s="27" t="n">
+        <v>357</v>
+      </c>
+      <c r="F6" s="27" t="s">
         <v>65</v>
       </c>
-      <c r="R3" s="28" t="s">
+      <c r="G6" s="27" t="s">
+        <v>66</v>
+      </c>
+      <c r="H6" s="28" t="n">
+        <v>42605</v>
+      </c>
+      <c r="I6" s="27" t="s">
+        <v>83</v>
+      </c>
+      <c r="K6" s="27" t="s">
+        <v>84</v>
+      </c>
+      <c r="L6" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="S3" s="28" t="s">
+      <c r="N6" s="27" t="s">
+        <v>85</v>
+      </c>
+      <c r="O6" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q6" s="27" t="s">
+        <v>67</v>
+      </c>
+      <c r="R6" s="27" t="s">
+        <v>69</v>
+      </c>
+      <c r="S6" s="27" t="s">
         <v>54</v>
       </c>
-      <c r="T3" s="28" t="s">
+      <c r="T6" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="X3" s="29" t="n">
-        <v>42993</v>
-      </c>
-      <c r="Y3" s="28" t="s">
-        <v>68</v>
-      </c>
-      <c r="AC3" s="28"/>
-      <c r="AD3" s="28" t="s">
+      <c r="Y6" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="AC6" s="27" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" s="27" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="27" t="s">
+        <v>80</v>
+      </c>
+      <c r="L7" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="N7" s="27" t="s">
+        <v>85</v>
+      </c>
+      <c r="Q7" s="27" t="s">
+        <v>67</v>
+      </c>
+      <c r="R7" s="27" t="s">
         <v>69</v>
       </c>
-      <c r="AJ3" s="31" t="s">
+      <c r="S7" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="T7" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="Y7" s="27" t="s">
+        <v>86</v>
+      </c>
+      <c r="AD7" s="27" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>88</v>
+      </c>
+      <c r="B8" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="C8" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8" s="0" t="n">
+        <v>582</v>
+      </c>
+      <c r="F8" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H8" s="31" t="n">
+        <v>38520</v>
+      </c>
+      <c r="I8" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="J8" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="O8" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="Q8" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="R8" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="S8" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="T8" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="V8" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="X8" s="31" t="s">
+        <v>101</v>
+      </c>
+      <c r="Y8" s="0" t="s">
         <v>70</v>
       </c>
-      <c r="AK3" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL3" s="28" t="s">
-        <v>72</v>
-      </c>
-      <c r="AM3" s="28" t="s">
-        <v>73</v>
+      <c r="Z8" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="AA8" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="AC8" s="1" t="s">
+        <v>60</v>
       </c>
     </row>
-    <row r="4" s="31" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="31" t="s">
-        <v>74</v>
-      </c>
-      <c r="AJ4" s="31" t="s">
-        <v>70</v>
-      </c>
-      <c r="AK4" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL4" s="28" t="s">
-        <v>75</v>
-      </c>
-      <c r="AM4" s="28" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="5" s="31" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="31" t="s">
-        <v>74</v>
-      </c>
-      <c r="AJ5" s="31" t="s">
-        <v>70</v>
-      </c>
-      <c r="AK5" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL5" s="28" t="s">
-        <v>77</v>
-      </c>
-      <c r="AM5" s="28" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="6" s="31" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="31" t="s">
-        <v>79</v>
-      </c>
-      <c r="B6" s="31" t="n">
-        <v>45.685327</v>
-      </c>
-      <c r="C6" s="31" t="n">
-        <v>13.833536</v>
-      </c>
-      <c r="D6" s="31" t="s">
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" s="0" t="s">
         <v>44</v>
       </c>
-      <c r="E6" s="31" t="n">
-        <v>357</v>
-      </c>
-      <c r="F6" s="31" t="s">
-        <v>63</v>
-      </c>
-      <c r="G6" s="28" t="s">
-        <v>64</v>
-      </c>
-      <c r="H6" s="29" t="n">
-        <v>42605</v>
-      </c>
-      <c r="I6" s="28" t="s">
-        <v>80</v>
-      </c>
-      <c r="K6" s="31" t="s">
-        <v>81</v>
-      </c>
-      <c r="L6" s="28" t="s">
-        <v>65</v>
-      </c>
-      <c r="M6" s="28"/>
-      <c r="N6" s="28" t="s">
-        <v>82</v>
-      </c>
-      <c r="O6" s="31" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q6" s="28" t="s">
-        <v>65</v>
-      </c>
-      <c r="R6" s="28" t="s">
-        <v>67</v>
-      </c>
-      <c r="S6" s="28" t="s">
+      <c r="E9" s="0" t="n">
+        <v>651</v>
+      </c>
+      <c r="F9" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="H9" s="31" t="n">
+        <v>30706</v>
+      </c>
+      <c r="I9" s="0" t="s">
+        <v>108</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="O9" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="Q9" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="R9" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="S9" s="0" t="s">
         <v>54</v>
       </c>
-      <c r="T6" s="28" t="s">
-        <v>55</v>
-      </c>
-      <c r="Y6" s="28" t="s">
-        <v>68</v>
-      </c>
-      <c r="AC6" s="28" t="s">
-        <v>60</v>
-      </c>
-      <c r="AD6" s="28"/>
-    </row>
-    <row r="7" s="31" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="31" t="s">
-        <v>79</v>
-      </c>
-      <c r="G7" s="28"/>
-      <c r="L7" s="28" t="s">
-        <v>54</v>
-      </c>
-      <c r="M7" s="28"/>
-      <c r="N7" s="28" t="s">
-        <v>82</v>
-      </c>
-      <c r="Q7" s="28" t="s">
-        <v>65</v>
-      </c>
-      <c r="R7" s="28" t="s">
-        <v>67</v>
-      </c>
-      <c r="S7" s="28" t="s">
-        <v>54</v>
-      </c>
-      <c r="T7" s="28" t="s">
-        <v>55</v>
-      </c>
-      <c r="Y7" s="31" t="s">
-        <v>83</v>
-      </c>
-      <c r="AC7" s="28"/>
-      <c r="AD7" s="28" t="s">
-        <v>84</v>
+      <c r="T9" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="X9" s="31" t="n">
+        <v>30706</v>
+      </c>
+      <c r="Y9" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="Z9" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="AA9" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="AE9" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="AF9" s="0" t="n">
+        <v>2003</v>
+      </c>
+      <c r="AG9" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="AI9" s="33" t="s">
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: added some examples with docs
</commit_message>
<xml_diff>
--- a/template/public/template.xlsx
+++ b/template/public/template.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="149">
   <si>
     <t xml:space="preserve">site_code</t>
   </si>
@@ -362,7 +362,7 @@
     <t xml:space="preserve">Hyporheic zone</t>
   </si>
   <si>
-    <t xml:space="preserve">Proasellus aff. Escolai</t>
+    <t xml:space="preserve">Proasellus aff. escolai</t>
   </si>
   <si>
     <t xml:space="preserve">Henry, J P</t>
@@ -378,6 +378,96 @@
   </si>
   <si>
     <t xml:space="preserve">Henry J.-P., Magniez G. 2003. Isopodes aselloides stygobies d Espagne, III - Le genre Proasellus: B - Especes anophtalmes. Beaufortia, 53(6), 129-158.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EGCop_375</t>
+  </si>
+  <si>
+    <t xml:space="preserve">43.02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.347</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;10km</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FRA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aquatic, Subsurface, Aquifer, Freshwater</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Graeteriella (Paragraeteriella)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subgenus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cyclopidae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Graeteriella</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PASCALIS Database</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lescher-Moutoué F.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personal communication</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CROATI06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">44.2585</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15.6629</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HRV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proasellus anophtalmus aff. rhausinus form A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proasellus anophtalmus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sket B.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sket B. 1965. Subterrane Asellus-Arten Jugoslaviens (Crustacea, Isopoda). Acta Musei Macedonici Scientiarum Naturalium, X(1), 1-26.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EGCop_1360</t>
+  </si>
+  <si>
+    <t xml:space="preserve">49.335</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.688</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diacyclops sp.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Genus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">group languidoides</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1111/j.1574-6941.2009.00674.x</t>
   </si>
 </sst>
 </file>
@@ -467,6 +557,7 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="7">
@@ -541,7 +632,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -662,15 +753,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -930,19 +1017,20 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AO9"/>
+  <dimension ref="A1:AO12"/>
   <sheetFormatPr defaultColWidth="16.96484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="35.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="23.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="28.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="1" width="42.69"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="28.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="49.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="19.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="1" width="22.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="1" width="24.2"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="1" width="34.49"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="1" width="25.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="0" width="19.27"/>
   </cols>
   <sheetData>
     <row r="1" s="26" customFormat="true" ht="29.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1332,34 +1420,34 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B8" s="30" t="s">
+      <c r="B8" s="29" t="s">
         <v>89</v>
       </c>
-      <c r="C8" s="30" t="s">
+      <c r="C8" s="29" t="s">
         <v>90</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="E8" s="0" t="n">
+      <c r="E8" s="1" t="n">
         <v>582</v>
       </c>
-      <c r="F8" s="0" t="s">
+      <c r="F8" s="1" t="s">
         <v>91</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="H8" s="31" t="n">
+      <c r="H8" s="30" t="n">
         <v>38520</v>
       </c>
-      <c r="I8" s="0" t="s">
+      <c r="I8" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="J8" s="0" t="s">
+      <c r="J8" s="1" t="s">
         <v>94</v>
       </c>
       <c r="K8" s="1" t="s">
@@ -1371,28 +1459,28 @@
       <c r="N8" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="O8" s="0" t="s">
+      <c r="O8" s="1" t="s">
         <v>97</v>
       </c>
       <c r="Q8" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="R8" s="0" t="s">
+      <c r="R8" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="S8" s="0" t="s">
+      <c r="S8" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="T8" s="0" t="s">
+      <c r="T8" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="V8" s="0" t="s">
+      <c r="V8" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="X8" s="31" t="s">
+      <c r="X8" s="30" t="s">
         <v>101</v>
       </c>
-      <c r="Y8" s="0" t="s">
+      <c r="Y8" s="1" t="s">
         <v>70</v>
       </c>
       <c r="Z8" s="1" t="s">
@@ -1406,31 +1494,31 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="E9" s="0" t="n">
+      <c r="E9" s="1" t="n">
         <v>651</v>
       </c>
-      <c r="F9" s="0" t="s">
+      <c r="F9" s="1" t="s">
         <v>91</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="H9" s="31" t="n">
+      <c r="H9" s="30" t="n">
         <v>30706</v>
       </c>
-      <c r="I9" s="0" t="s">
+      <c r="I9" s="1" t="s">
         <v>108</v>
       </c>
       <c r="K9" s="1" t="s">
@@ -1442,25 +1530,25 @@
       <c r="N9" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="O9" s="0" t="s">
+      <c r="O9" s="1" t="s">
         <v>112</v>
       </c>
       <c r="Q9" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="R9" s="0" t="s">
+      <c r="R9" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="S9" s="0" t="s">
+      <c r="S9" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="T9" s="0" t="s">
+      <c r="T9" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="X9" s="31" t="n">
+      <c r="X9" s="30" t="n">
         <v>30706</v>
       </c>
-      <c r="Y9" s="0" t="s">
+      <c r="Y9" s="1" t="s">
         <v>114</v>
       </c>
       <c r="Z9" s="1" t="s">
@@ -1469,17 +1557,146 @@
       <c r="AA9" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="AE9" s="0" t="s">
+      <c r="AE9" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="AF9" s="0" t="n">
+      <c r="AF9" s="1" t="n">
         <v>2003</v>
       </c>
-      <c r="AG9" s="32" t="s">
+      <c r="AG9" s="31" t="s">
         <v>117</v>
       </c>
-      <c r="AI9" s="33" t="s">
+      <c r="AI9" s="32" t="s">
         <v>118</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="C10" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="D10" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="F10" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="O10" s="0" t="s">
+        <v>125</v>
+      </c>
+      <c r="Q10" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="R10" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="S10" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="T10" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="AC10" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="AE10" s="0" t="s">
+        <v>131</v>
+      </c>
+      <c r="AF10" s="0" t="n">
+        <v>2005</v>
+      </c>
+      <c r="AG10" s="0" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
+        <v>133</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>134</v>
+      </c>
+      <c r="C11" s="0" t="s">
+        <v>135</v>
+      </c>
+      <c r="D11" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="F11" s="0" t="s">
+        <v>136</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q11" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="R11" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="S11" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="T11" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="U11" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="AE11" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="AF11" s="0" t="n">
+        <v>1965</v>
+      </c>
+      <c r="AI11" s="0" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>142</v>
+      </c>
+      <c r="C12" s="0" t="s">
+        <v>143</v>
+      </c>
+      <c r="D12" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="F12" s="0" t="s">
+        <v>144</v>
+      </c>
+      <c r="N12" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q12" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="R12" s="0" t="s">
+        <v>146</v>
+      </c>
+      <c r="S12" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="W12" s="0" t="s">
+        <v>147</v>
+      </c>
+      <c r="AD12" s="1" t="s">
+        <v>148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: more improvements on import template and docs
</commit_message>
<xml_diff>
--- a/template/public/template.xlsx
+++ b/template/public/template.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="169">
   <si>
     <t xml:space="preserve">site_code</t>
   </si>
@@ -143,12 +143,42 @@
     <t xml:space="preserve">sequence_content</t>
   </si>
   <si>
-    <t xml:space="preserve">sampling_effort</t>
+    <t xml:space="preserve">site_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">site_comments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sampling_duration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sampling_comments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">unclassified</t>
+  </si>
+  <si>
+    <t xml:space="preserve">specific_epithet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">occurrence_comments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">collection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sequence_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">seq_comments</t>
   </si>
   <si>
     <t xml:space="preserve">PIVKACAV</t>
   </si>
   <si>
+    <t xml:space="preserve">Planina cave,  Pivka channel</t>
+  </si>
+  <si>
     <t xml:space="preserve">45.819984</t>
   </si>
   <si>
@@ -191,19 +221,16 @@
     <t xml:space="preserve">Asellus</t>
   </si>
   <si>
-    <t xml:space="preserve">Asellus aquaticus</t>
+    <t xml:space="preserve">aquaticus</t>
   </si>
   <si>
     <t xml:space="preserve">Prevorcnik, Simona</t>
   </si>
   <si>
-    <t xml:space="preserve">Ten</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15 specimens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">World Asellidae Database</t>
+    <t xml:space="preserve">World Asellidae Database[int:1787]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UCBLZ</t>
   </si>
   <si>
     <t xml:space="preserve">10.1127/0003-9136/2004/0160-0193</t>
@@ -212,6 +239,9 @@
     <t xml:space="preserve">MERAVIGL</t>
   </si>
   <si>
+    <t xml:space="preserve">Grotta Meravigliosa Di Lazzaro Jerko Opicina Italy</t>
+  </si>
+  <si>
     <t xml:space="preserve">45.688</t>
   </si>
   <si>
@@ -233,15 +263,24 @@
     <t xml:space="preserve">Species</t>
   </si>
   <si>
+    <t xml:space="preserve">kosswigi</t>
+  </si>
+  <si>
     <t xml:space="preserve">Malard, Florian</t>
   </si>
   <si>
+    <t xml:space="preserve">Several</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MERAVIGL_Akosswigi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">World Asellidae Database[ext:3990]</t>
+  </si>
+  <si>
     <t xml:space="preserve">10.1002/eco.1727</t>
   </si>
   <si>
-    <t xml:space="preserve">MERAVIGL_Akosswigi</t>
-  </si>
-  <si>
     <t xml:space="preserve">COI</t>
   </si>
   <si>
@@ -266,6 +305,9 @@
     <t xml:space="preserve">TREBICGR</t>
   </si>
   <si>
+    <t xml:space="preserve">Trebiciano cave</t>
+  </si>
+  <si>
     <t xml:space="preserve">45.685327</t>
   </si>
   <si>
@@ -281,15 +323,24 @@
     <t xml:space="preserve">Aquatic, Subsurface, Aquifer, Karst</t>
   </si>
   <si>
+    <t xml:space="preserve">World Asellidae Database[int:83]</t>
+  </si>
+  <si>
     <t xml:space="preserve">Verovnik, R</t>
   </si>
   <si>
+    <t xml:space="preserve">World Asellidae Database[ext:4006]</t>
+  </si>
+  <si>
     <t xml:space="preserve">10.1016/j.jcz.2009.03.001</t>
   </si>
   <si>
     <t xml:space="preserve">SIPANFON</t>
   </si>
   <si>
+    <t xml:space="preserve">Fontaine Rio Guatizalema Puente Cerca Sipan</t>
+  </si>
+  <si>
     <t xml:space="preserve">42.1831</t>
   </si>
   <si>
@@ -323,21 +374,24 @@
     <t xml:space="preserve">Proasellus</t>
   </si>
   <si>
+    <t xml:space="preserve">lescherae</t>
+  </si>
+  <si>
     <t xml:space="preserve">true</t>
   </si>
   <si>
     <t xml:space="preserve">2010-01</t>
   </si>
   <si>
-    <t xml:space="preserve">Several</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3 specimens</t>
+    <t xml:space="preserve">World Asellidae Database[int:6077]</t>
   </si>
   <si>
     <t xml:space="preserve">GUADALQ1</t>
   </si>
   <si>
+    <t xml:space="preserve">Rio Guadalquivir Coto Rìos</t>
+  </si>
+  <si>
     <t xml:space="preserve">38.0628</t>
   </si>
   <si>
@@ -365,12 +419,18 @@
     <t xml:space="preserve">Proasellus aff. escolai</t>
   </si>
   <si>
+    <t xml:space="preserve">escolai</t>
+  </si>
+  <si>
     <t xml:space="preserve">Henry, J P</t>
   </si>
   <si>
     <t xml:space="preserve">8 juveniles</t>
   </si>
   <si>
+    <t xml:space="preserve">World Asellidae Database[ext:394]</t>
+  </si>
+  <si>
     <t xml:space="preserve">Henry J.-P., Magniez G.</t>
   </si>
   <si>
@@ -380,7 +440,7 @@
     <t xml:space="preserve">Henry J.-P., Magniez G. 2003. Isopodes aselloides stygobies d Espagne, III - Le genre Proasellus: B - Especes anophtalmes. Beaufortia, 53(6), 129-158.</t>
   </si>
   <si>
-    <t xml:space="preserve">EGCop_375</t>
+    <t xml:space="preserve">Durban-sur-Arize, source</t>
   </si>
   <si>
     <t xml:space="preserve">43.02</t>
@@ -437,16 +497,16 @@
     <t xml:space="preserve">Proasellus anophtalmus aff. rhausinus form A</t>
   </si>
   <si>
-    <t xml:space="preserve">Proasellus anophtalmus</t>
+    <t xml:space="preserve">anophtalmus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">World Asellidae Database[ext:2078]</t>
   </si>
   <si>
     <t xml:space="preserve">Sket B.</t>
   </si>
   <si>
     <t xml:space="preserve">Sket B. 1965. Subterrane Asellus-Arten Jugoslaviens (Crustacea, Isopoda). Acta Musei Macedonici Scientiarum Naturalium, X(1), 1-26.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EGCop_1360</t>
   </si>
   <si>
     <t xml:space="preserve">49.335</t>
@@ -474,9 +534,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="166" formatCode="0"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -532,7 +593,6 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
-      <color rgb="FFF10D0C"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -540,6 +600,7 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
+      <color rgb="FFF10D0C"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -560,7 +621,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -593,8 +654,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF8C0C0"/>
+        <bgColor rgb="FFF4C0F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFD7"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4C0F8"/>
+        <bgColor rgb="FFF8C0C0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE699"/>
+        <bgColor rgb="FFFFFFD7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFD9D9D9"/>
-        <bgColor rgb="FFCCFFCC"/>
+        <bgColor rgb="FFF4C0F8"/>
       </patternFill>
     </fill>
   </fills>
@@ -632,7 +717,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="36">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -701,7 +786,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -709,23 +794,19 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -733,7 +814,15 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -745,6 +834,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="11" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -757,11 +850,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="11" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -794,7 +891,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF729FCF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFFFFFD7"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -811,11 +908,11 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FFFFE699"/>
       <rgbColor rgb="FF97C7A6"/>
-      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFF4C0F8"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFF8C0C0"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -1017,686 +1114,783 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AO12"/>
+  <dimension ref="A1:AW12"/>
   <sheetFormatPr defaultColWidth="16.96484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="35.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="23.36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="28.65"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="1" width="42.69"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="49.65"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="19.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="1" width="22.39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="1" width="24.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="1" width="34.49"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="1" width="25.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="0" width="19.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="35.05"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="16.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="23.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="28.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="1" width="42.69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="49.65"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="16.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="1" width="19.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="1" width="22.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="0" width="24.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="34" style="1" width="25.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="1" width="35.32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="1" width="73.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="1" width="34.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="43" style="1" width="25.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="48" min="48" style="1" width="19.27"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="49" min="49" style="1" width="16.96"/>
   </cols>
   <sheetData>
-    <row r="1" s="26" customFormat="true" ht="29.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" s="27" customFormat="true" ht="29.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="D1" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="E1" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="F1" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="G1" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="H1" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="17" t="s">
+      <c r="I1" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="J1" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="18" t="s">
+      <c r="K1" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="18" t="s">
+      <c r="L1" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="18" t="s">
+      <c r="M1" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="18" t="s">
+      <c r="N1" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="N1" s="17" t="s">
+      <c r="O1" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="P1" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="17" t="s">
+      <c r="Q1" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="18" t="s">
+      <c r="R1" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="S1" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="19" t="s">
+      <c r="T1" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="19" t="s">
+      <c r="U1" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="V1" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="S1" s="19" t="s">
+      <c r="W1" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="T1" s="19" t="s">
+      <c r="X1" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="U1" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="V1" s="21" t="s">
+      <c r="Y1" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z1" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="W1" s="21" t="s">
+      <c r="AA1" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="X1" s="21" t="s">
+      <c r="AB1" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="Y1" s="21" t="s">
+      <c r="AC1" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="Z1" s="22" t="s">
+      <c r="AD1" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="AA1" s="22" t="s">
+      <c r="AE1" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="AB1" s="22" t="s">
+      <c r="AF1" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="AC1" s="22" t="s">
+      <c r="AG1" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="AH1" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="AI1" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="AD1" s="23" t="s">
+      <c r="AJ1" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="AK1" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="AE1" s="24" t="s">
+      <c r="AL1" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="AF1" s="24" t="s">
+      <c r="AM1" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="AG1" s="24" t="s">
+      <c r="AN1" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="AH1" s="24" t="s">
+      <c r="AO1" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="AI1" s="24" t="s">
+      <c r="AP1" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="AJ1" s="22" t="s">
+      <c r="AQ1" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="AK1" s="22" t="s">
+      <c r="AR1" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="AL1" s="22" t="s">
+      <c r="AS1" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="AM1" s="22" t="s">
+      <c r="AT1" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="AN1" s="22" t="s">
+      <c r="AU1" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="AO1" s="25" t="s">
-        <v>39</v>
+      <c r="AV1" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="AW1" s="26" t="s">
+        <v>49</v>
       </c>
     </row>
-    <row r="2" s="27" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="27" t="s">
-        <v>41</v>
-      </c>
-      <c r="B2" s="27" t="s">
-        <v>42</v>
-      </c>
-      <c r="C2" s="27" t="s">
-        <v>43</v>
-      </c>
-      <c r="D2" s="27" t="s">
-        <v>44</v>
-      </c>
-      <c r="E2" s="27" t="n">
+    <row r="2" s="28" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="D2" s="28" t="s">
+        <v>53</v>
+      </c>
+      <c r="E2" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="F2" s="28" t="n">
         <v>526</v>
       </c>
-      <c r="F2" s="27" t="s">
-        <v>45</v>
-      </c>
-      <c r="G2" s="27" t="s">
-        <v>46</v>
-      </c>
-      <c r="H2" s="28" t="n">
+      <c r="G2" s="28" t="s">
+        <v>55</v>
+      </c>
+      <c r="H2" s="28" t="s">
+        <v>56</v>
+      </c>
+      <c r="J2" s="30" t="n">
         <v>34023</v>
       </c>
-      <c r="I2" s="27" t="s">
-        <v>47</v>
-      </c>
-      <c r="J2" s="27" t="s">
-        <v>48</v>
-      </c>
-      <c r="K2" s="27" t="s">
-        <v>49</v>
-      </c>
-      <c r="L2" s="27" t="s">
-        <v>50</v>
-      </c>
-      <c r="N2" s="27" t="s">
-        <v>51</v>
-      </c>
-      <c r="O2" s="27" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q2" s="27" t="s">
-        <v>50</v>
-      </c>
-      <c r="R2" s="27" t="s">
-        <v>53</v>
-      </c>
-      <c r="S2" s="27" t="s">
+      <c r="K2" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="L2" s="28" t="s">
+        <v>58</v>
+      </c>
+      <c r="M2" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="N2" s="28" t="s">
+        <v>60</v>
+      </c>
+      <c r="P2" s="28" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q2" s="28" t="s">
+        <v>62</v>
+      </c>
+      <c r="T2" s="28" t="s">
+        <v>60</v>
+      </c>
+      <c r="V2" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="W2" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="X2" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y2" s="28" t="s">
+        <v>66</v>
+      </c>
+      <c r="AB2" s="30" t="n">
+        <v>34023</v>
+      </c>
+      <c r="AC2" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD2" s="28" t="n">
+        <v>15</v>
+      </c>
+      <c r="AI2" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="AJ2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="AK2" s="31" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" s="28" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>72</v>
+      </c>
+      <c r="C3" s="28" t="s">
+        <v>73</v>
+      </c>
+      <c r="D3" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="F3" s="28" t="n">
+        <v>322</v>
+      </c>
+      <c r="G3" s="28" t="s">
+        <v>75</v>
+      </c>
+      <c r="H3" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="N3" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="P3" s="28" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q3" s="28" t="s">
+        <v>62</v>
+      </c>
+      <c r="T3" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="V3" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="W3" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="X3" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y3" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="AB3" s="30" t="n">
+        <v>42993</v>
+      </c>
+      <c r="AC3" s="28" t="s">
+        <v>81</v>
+      </c>
+      <c r="AD3" s="28" t="s">
+        <v>82</v>
+      </c>
+      <c r="AH3" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="AI3" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="AK3" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="AQ3" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="AR3" s="28" t="s">
+        <v>86</v>
+      </c>
+      <c r="AS3" s="28" t="s">
+        <v>87</v>
+      </c>
+      <c r="AT3" s="28" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="4" s="28" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="AH4" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="AQ4" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="AR4" s="28" t="s">
+        <v>86</v>
+      </c>
+      <c r="AS4" s="28" t="s">
+        <v>89</v>
+      </c>
+      <c r="AT4" s="28" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" s="28" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="AH5" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="AQ5" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="AR5" s="28" t="s">
+        <v>86</v>
+      </c>
+      <c r="AS5" s="28" t="s">
+        <v>91</v>
+      </c>
+      <c r="AT5" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="6" s="28" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="28" t="s">
+        <v>93</v>
+      </c>
+      <c r="B6" s="29" t="s">
+        <v>94</v>
+      </c>
+      <c r="C6" s="28" t="s">
+        <v>95</v>
+      </c>
+      <c r="D6" s="28" t="s">
+        <v>96</v>
+      </c>
+      <c r="E6" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="T2" s="27" t="s">
-        <v>55</v>
-      </c>
-      <c r="U2" s="27" t="s">
-        <v>56</v>
-      </c>
-      <c r="X2" s="28" t="n">
-        <v>34023</v>
-      </c>
-      <c r="Y2" s="27" t="s">
-        <v>57</v>
-      </c>
-      <c r="Z2" s="27" t="s">
-        <v>58</v>
-      </c>
-      <c r="AA2" s="27" t="s">
+      <c r="F6" s="28" t="n">
+        <v>357</v>
+      </c>
+      <c r="G6" s="28" t="s">
+        <v>75</v>
+      </c>
+      <c r="H6" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="J6" s="30" t="n">
+        <v>42605</v>
+      </c>
+      <c r="K6" s="28" t="s">
+        <v>97</v>
+      </c>
+      <c r="M6" s="28" t="s">
+        <v>98</v>
+      </c>
+      <c r="N6" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="P6" s="28" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q6" s="28" t="s">
+        <v>62</v>
+      </c>
+      <c r="T6" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="V6" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="W6" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="X6" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y6" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="AC6" s="28" t="s">
+        <v>81</v>
+      </c>
+      <c r="AI6" s="28" t="s">
+        <v>100</v>
+      </c>
+      <c r="AJ6" s="28" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" s="28" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="28" t="s">
+        <v>93</v>
+      </c>
+      <c r="N7" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="P7" s="28" t="s">
+        <v>99</v>
+      </c>
+      <c r="T7" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="V7" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="W7" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="X7" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y7" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="AC7" s="28" t="s">
+        <v>101</v>
+      </c>
+      <c r="AI7" s="28" t="s">
+        <v>102</v>
+      </c>
+      <c r="AK7" s="28" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B8" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="C8" s="31" t="s">
+        <v>106</v>
+      </c>
+      <c r="D8" s="31" t="s">
+        <v>107</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>582</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="J8" s="32" t="n">
+        <v>38520</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="M8" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="AC2" s="27" t="s">
-        <v>60</v>
-      </c>
-      <c r="AD2" s="29" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="3" s="27" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="27" t="s">
-        <v>62</v>
-      </c>
-      <c r="B3" s="27" t="s">
-        <v>63</v>
-      </c>
-      <c r="C3" s="27" t="s">
+      <c r="N8" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="P8" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q8" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="R8" s="1"/>
+      <c r="T8" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="V8" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="W8" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="E3" s="27" t="n">
-        <v>322</v>
-      </c>
-      <c r="F3" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="G3" s="27" t="s">
-        <v>66</v>
-      </c>
-      <c r="L3" s="27" t="s">
-        <v>67</v>
-      </c>
-      <c r="N3" s="27" t="s">
-        <v>68</v>
-      </c>
-      <c r="O3" s="27" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q3" s="27" t="s">
-        <v>67</v>
-      </c>
-      <c r="R3" s="27" t="s">
+      <c r="X8" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="Y8" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="Z8" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="AB8" s="32" t="s">
+        <v>119</v>
+      </c>
+      <c r="AC8" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="AD8" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI8" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="AJ8" s="1" t="s">
         <v>69</v>
-      </c>
-      <c r="S3" s="27" t="s">
-        <v>54</v>
-      </c>
-      <c r="T3" s="27" t="s">
-        <v>55</v>
-      </c>
-      <c r="X3" s="28" t="n">
-        <v>42993</v>
-      </c>
-      <c r="Y3" s="27" t="s">
-        <v>70</v>
-      </c>
-      <c r="AD3" s="27" t="s">
-        <v>71</v>
-      </c>
-      <c r="AJ3" s="27" t="s">
-        <v>72</v>
-      </c>
-      <c r="AK3" s="27" t="s">
-        <v>73</v>
-      </c>
-      <c r="AL3" s="27" t="s">
-        <v>74</v>
-      </c>
-      <c r="AM3" s="27" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="4" s="27" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="27" t="s">
-        <v>62</v>
-      </c>
-      <c r="AJ4" s="27" t="s">
-        <v>72</v>
-      </c>
-      <c r="AK4" s="27" t="s">
-        <v>73</v>
-      </c>
-      <c r="AL4" s="27" t="s">
-        <v>76</v>
-      </c>
-      <c r="AM4" s="27" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="5" s="27" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="27" t="s">
-        <v>62</v>
-      </c>
-      <c r="AJ5" s="27" t="s">
-        <v>72</v>
-      </c>
-      <c r="AK5" s="27" t="s">
-        <v>73</v>
-      </c>
-      <c r="AL5" s="27" t="s">
-        <v>78</v>
-      </c>
-      <c r="AM5" s="27" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="6" s="27" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="B6" s="27" t="s">
-        <v>81</v>
-      </c>
-      <c r="C6" s="27" t="s">
-        <v>82</v>
-      </c>
-      <c r="D6" s="27" t="s">
-        <v>44</v>
-      </c>
-      <c r="E6" s="27" t="n">
-        <v>357</v>
-      </c>
-      <c r="F6" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="G6" s="27" t="s">
-        <v>66</v>
-      </c>
-      <c r="H6" s="28" t="n">
-        <v>42605</v>
-      </c>
-      <c r="I6" s="27" t="s">
-        <v>83</v>
-      </c>
-      <c r="K6" s="27" t="s">
-        <v>84</v>
-      </c>
-      <c r="L6" s="27" t="s">
-        <v>67</v>
-      </c>
-      <c r="N6" s="27" t="s">
-        <v>85</v>
-      </c>
-      <c r="O6" s="27" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q6" s="27" t="s">
-        <v>67</v>
-      </c>
-      <c r="R6" s="27" t="s">
-        <v>69</v>
-      </c>
-      <c r="S6" s="27" t="s">
-        <v>54</v>
-      </c>
-      <c r="T6" s="27" t="s">
-        <v>55</v>
-      </c>
-      <c r="Y6" s="27" t="s">
-        <v>70</v>
-      </c>
-      <c r="AC6" s="27" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="7" s="27" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="L7" s="27" t="s">
-        <v>54</v>
-      </c>
-      <c r="N7" s="27" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q7" s="27" t="s">
-        <v>67</v>
-      </c>
-      <c r="R7" s="27" t="s">
-        <v>69</v>
-      </c>
-      <c r="S7" s="27" t="s">
-        <v>54</v>
-      </c>
-      <c r="T7" s="27" t="s">
-        <v>55</v>
-      </c>
-      <c r="Y7" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="AD7" s="27" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B8" s="29" t="s">
-        <v>89</v>
-      </c>
-      <c r="C8" s="29" t="s">
-        <v>90</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E8" s="1" t="n">
-        <v>582</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="H8" s="30" t="n">
-        <v>38520</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="L8" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="N8" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="O8" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="Q8" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="R8" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="S8" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="T8" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="V8" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="X8" s="30" t="s">
-        <v>101</v>
-      </c>
-      <c r="Y8" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="Z8" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="AA8" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="AC8" s="1" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>105</v>
+        <v>121</v>
+      </c>
+      <c r="B9" s="33" t="s">
+        <v>122</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>106</v>
+        <v>123</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E9" s="1" t="n">
+        <v>124</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F9" s="1" t="n">
         <v>651</v>
       </c>
-      <c r="F9" s="1" t="s">
-        <v>91</v>
-      </c>
       <c r="G9" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="H9" s="30" t="n">
+        <v>108</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="J9" s="32" t="n">
         <v>30706</v>
       </c>
-      <c r="I9" s="1" t="s">
-        <v>108</v>
-      </c>
       <c r="K9" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="L9" s="1" t="s">
-        <v>110</v>
+        <v>126</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>127</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="O9" s="1" t="s">
-        <v>112</v>
+        <v>128</v>
+      </c>
+      <c r="P9" s="1" t="s">
+        <v>129</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="R9" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="S9" s="1" t="s">
-        <v>54</v>
-      </c>
+        <v>130</v>
+      </c>
+      <c r="R9" s="1"/>
       <c r="T9" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="X9" s="30" t="n">
+        <v>131</v>
+      </c>
+      <c r="U9" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="V9" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="W9" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="X9" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="Y9" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="AB9" s="32" t="n">
         <v>30706</v>
       </c>
-      <c r="Y9" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="Z9" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="AA9" s="1" t="s">
-        <v>115</v>
+      <c r="AC9" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="AD9" s="1" t="n">
+        <v>8</v>
       </c>
       <c r="AE9" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="AF9" s="1" t="n">
+        <v>134</v>
+      </c>
+      <c r="AI9" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="AL9" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="AM9" s="1" t="n">
         <v>2003</v>
       </c>
-      <c r="AG9" s="31" t="s">
-        <v>117</v>
-      </c>
-      <c r="AI9" s="32" t="s">
-        <v>118</v>
+      <c r="AN9" s="34" t="s">
+        <v>137</v>
+      </c>
+      <c r="AP9" s="35" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
-        <v>119</v>
-      </c>
+      <c r="A10" s="1"/>
       <c r="B10" s="0" t="s">
-        <v>120</v>
-      </c>
-      <c r="C10" s="0" t="s">
-        <v>121</v>
-      </c>
-      <c r="D10" s="0" t="s">
-        <v>122</v>
-      </c>
-      <c r="F10" s="0" t="s">
-        <v>123</v>
-      </c>
-      <c r="N10" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="O10" s="0" t="s">
-        <v>125</v>
+        <v>139</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="P10" s="1" t="s">
+        <v>144</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="R10" s="0" t="s">
-        <v>127</v>
-      </c>
-      <c r="S10" s="0" t="s">
-        <v>128</v>
-      </c>
-      <c r="T10" s="0" t="s">
-        <v>129</v>
-      </c>
-      <c r="AC10" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="AE10" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="AF10" s="0" t="n">
+        <v>145</v>
+      </c>
+      <c r="R10" s="1"/>
+      <c r="T10" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="V10" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="W10" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="X10" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="AI10" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="AL10" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="AM10" s="1" t="n">
         <v>2005</v>
       </c>
-      <c r="AG10" s="0" t="s">
-        <v>132</v>
+      <c r="AN10" s="1" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
-        <v>133</v>
-      </c>
-      <c r="B11" s="0" t="s">
-        <v>134</v>
-      </c>
-      <c r="C11" s="0" t="s">
-        <v>135</v>
-      </c>
-      <c r="D11" s="0" t="s">
-        <v>122</v>
-      </c>
-      <c r="F11" s="0" t="s">
-        <v>136</v>
-      </c>
-      <c r="L11" s="1" t="s">
-        <v>99</v>
+      <c r="A11" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>156</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="Q11" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="R11" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="S11" s="0" t="s">
-        <v>54</v>
-      </c>
-      <c r="T11" s="0" t="s">
-        <v>99</v>
-      </c>
-      <c r="U11" s="0" t="s">
-        <v>138</v>
-      </c>
-      <c r="AE11" s="0" t="s">
-        <v>139</v>
-      </c>
-      <c r="AF11" s="0" t="n">
+        <v>116</v>
+      </c>
+      <c r="P11" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="T11" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="U11" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="V11" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="W11" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="X11" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="Y11" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="AI11" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="AL11" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="AM11" s="1" t="n">
         <v>1965</v>
       </c>
-      <c r="AI11" s="0" t="s">
-        <v>140</v>
+      <c r="AP11" s="1" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
-        <v>141</v>
-      </c>
-      <c r="B12" s="0" t="s">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="C12" s="0" t="s">
-        <v>143</v>
-      </c>
-      <c r="D12" s="0" t="s">
-        <v>122</v>
-      </c>
-      <c r="F12" s="0" t="s">
-        <v>144</v>
-      </c>
-      <c r="N12" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="Q12" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="R12" s="0" t="s">
-        <v>146</v>
-      </c>
-      <c r="S12" s="0" t="s">
-        <v>128</v>
-      </c>
-      <c r="W12" s="0" t="s">
-        <v>147</v>
-      </c>
-      <c r="AD12" s="1" t="s">
+      <c r="G12" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="P12" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="T12" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="V12" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="W12" s="1" t="s">
         <v>148</v>
+      </c>
+      <c r="AA12" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK12" s="1" t="s">
+        <v>168</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: updated template wrt to guidelines and examples
</commit_message>
<xml_diff>
--- a/template/public/template.xlsx
+++ b/template/public/template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,11 +21,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="167">
   <si>
     <t xml:space="preserve">site_code</t>
   </si>
   <si>
+    <t xml:space="preserve">site_name</t>
+  </si>
+  <si>
     <t xml:space="preserve">latitude</t>
   </si>
   <si>
@@ -44,6 +47,9 @@
     <t xml:space="preserve">locality</t>
   </si>
   <si>
+    <t xml:space="preserve">site_comments</t>
+  </si>
+  <si>
     <t xml:space="preserve">sampling_date</t>
   </si>
   <si>
@@ -65,12 +71,18 @@
     <t xml:space="preserve">access_points</t>
   </si>
   <si>
+    <t xml:space="preserve">sampling_comments</t>
+  </si>
+  <si>
     <t xml:space="preserve">sampling_id</t>
   </si>
   <si>
     <t xml:space="preserve">taxon_name</t>
   </si>
   <si>
+    <t xml:space="preserve">unclassified</t>
+  </si>
+  <si>
     <t xml:space="preserve">taxon_rank</t>
   </si>
   <si>
@@ -80,7 +92,7 @@
     <t xml:space="preserve">genus</t>
   </si>
   <si>
-    <t xml:space="preserve">species</t>
+    <t xml:space="preserve">specific_epithet</t>
   </si>
   <si>
     <t xml:space="preserve">tax_id_confer</t>
@@ -104,9 +116,18 @@
     <t xml:space="preserve">type_status</t>
   </si>
   <si>
+    <t xml:space="preserve">occurrence_comments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">occurrence_id</t>
+  </si>
+  <si>
     <t xml:space="preserve">data_repository</t>
   </si>
   <si>
+    <t xml:space="preserve">collection</t>
+  </si>
+  <si>
     <t xml:space="preserve">pub_DOI</t>
   </si>
   <si>
@@ -125,9 +146,6 @@
     <t xml:space="preserve">pub_verbatim</t>
   </si>
   <si>
-    <t xml:space="preserve">occurrence_id</t>
-  </si>
-  <si>
     <t xml:space="preserve">gene</t>
   </si>
   <si>
@@ -140,37 +158,13 @@
     <t xml:space="preserve">MOTU</t>
   </si>
   <si>
-    <t xml:space="preserve">sequence_content</t>
-  </si>
-  <si>
-    <t xml:space="preserve">site_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">site_comments</t>
+    <t xml:space="preserve">sequence_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">seq_comments</t>
   </si>
   <si>
     <t xml:space="preserve">sampling_duration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sampling_comments</t>
-  </si>
-  <si>
-    <t xml:space="preserve">unclassified</t>
-  </si>
-  <si>
-    <t xml:space="preserve">specific_epithet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">occurrence_comments</t>
-  </si>
-  <si>
-    <t xml:space="preserve">collection</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sequence_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">seq_comments</t>
   </si>
   <si>
     <t xml:space="preserve">PIVKACAV</t>
@@ -564,7 +558,6 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
-      <color rgb="FFF10D0C"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -572,6 +565,7 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
+      <color rgb="FFF10D0C"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -648,26 +642,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFD7"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF729FCF"/>
         <bgColor rgb="FF969696"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF8C0C0"/>
-        <bgColor rgb="FFF4C0F8"/>
+        <fgColor rgb="FFF4C0F8"/>
+        <bgColor rgb="FFF8C0C0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFD7"/>
-        <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF4C0F8"/>
-        <bgColor rgb="FFF8C0C0"/>
+        <fgColor rgb="FFF8C0C0"/>
+        <bgColor rgb="FFF4C0F8"/>
       </patternFill>
     </fill>
     <fill>
@@ -717,7 +711,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -738,7 +732,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -750,7 +744,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -758,22 +752,34 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -794,7 +800,23 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -802,28 +824,8 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -939,66 +941,66 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AT1"/>
+  <dimension ref="A1:BA1"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15.43"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="7" min="5" style="1" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="14.6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="20.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="19.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="17.94"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="17.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="13.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="14.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="15.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="13.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="13.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="19" style="1" width="14.6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="20.16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="23" style="1" width="16.69"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="18.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="1" width="19.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="1" width="16.69"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="1" width="20.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="33" style="1" width="13.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="1" width="14.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="1" width="21.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="1" width="20.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="1" width="19.47"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15.43"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="6" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="1" width="14.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="20.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="19.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="17.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="17.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="13.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="14.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="17" style="1" width="15.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="13.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="20" style="1" width="13.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="23" style="1" width="14.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="20.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="27" style="1" width="16.69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="1" width="18.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="1" width="19.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="1" width="33.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="33" style="1" width="16.69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="35" style="1" width="20.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="40" style="1" width="13.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="43" style="1" width="26.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="1" width="20.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="46" min="46" style="1" width="19.47"/>
   </cols>
   <sheetData>
-    <row r="1" s="10" customFormat="true" ht="29.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" s="16" customFormat="true" ht="29.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
       <c r="K1" s="6" t="s">
@@ -1007,96 +1009,117 @@
       <c r="L1" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="M1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="N1" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="O1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="7" t="s">
+      <c r="P1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="7" t="s">
+      <c r="Q1" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="7" t="s">
+      <c r="R1" s="6" t="s">
         <v>17</v>
       </c>
       <c r="S1" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="8" t="s">
+      <c r="T1" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="9" t="s">
+      <c r="U1" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="9" t="s">
+      <c r="V1" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="9" t="s">
+      <c r="W1" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="9" t="s">
+      <c r="X1" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="10" t="s">
+      <c r="Y1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="10" t="s">
+      <c r="Z1" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="10" t="s">
+      <c r="AA1" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="10" t="s">
+      <c r="AB1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="11" t="s">
+      <c r="AC1" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="12" t="s">
+      <c r="AD1" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="12" t="s">
+      <c r="AE1" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="12" t="s">
+      <c r="AF1" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="12" t="s">
+      <c r="AG1" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="12" t="s">
+      <c r="AH1" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" s="10" t="s">
+      <c r="AI1" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" s="10" t="s">
+      <c r="AJ1" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" s="10" t="s">
+      <c r="AK1" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" s="10" t="s">
+      <c r="AL1" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" s="10" t="s">
+      <c r="AM1" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" s="13" t="s">
+      <c r="AN1" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" s="1"/>
-      <c r="AP1" s="1"/>
-      <c r="AQ1" s="1"/>
-      <c r="AR1" s="1"/>
-      <c r="AS1" s="1"/>
-      <c r="AT1" s="1"/>
+      <c r="AO1" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP1" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="AQ1" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="AR1" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="AS1" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="AT1" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="AU1" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="AV1" s="1"/>
+      <c r="AW1" s="1"/>
+      <c r="AX1" s="1"/>
+      <c r="AY1" s="1"/>
+      <c r="AZ1" s="1"/>
+      <c r="BA1" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1126,771 +1149,766 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="16.96"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="1" width="19.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="1" width="22.39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="0" width="24.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="1" width="24.2"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="34" style="1" width="25.04"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="1" width="35.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="1" width="73.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="1" width="34.49"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="43" style="1" width="25.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="48" min="48" style="1" width="19.27"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="49" min="49" style="1" width="16.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="47" min="47" style="1" width="19.27"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="48" min="48" style="1" width="16.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
   </cols>
   <sheetData>
-    <row r="1" s="27" customFormat="true" ht="29.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+    <row r="1" s="29" customFormat="true" ht="29.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="P1" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q1" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="S1" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="T1" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="U1" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="V1" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="W1" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="X1" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y1" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="Z1" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="AA1" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB1" s="24" t="s">
+        <v>26</v>
+      </c>
+      <c r="AC1" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="AD1" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="AE1" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="AF1" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="AG1" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="AH1" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="AI1" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="AJ1" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="AK1" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="AL1" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="AM1" s="26" t="s">
+        <v>37</v>
+      </c>
+      <c r="AN1" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="AO1" s="26" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP1" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="C1" s="16" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="14" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="14" t="s">
+      <c r="AQ1" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="J1" s="17" t="s">
-        <v>7</v>
-      </c>
-      <c r="K1" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="L1" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="M1" s="18" t="s">
-        <v>10</v>
-      </c>
-      <c r="N1" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="O1" s="18" t="s">
+      <c r="AR1" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="P1" s="17" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q1" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="R1" s="18" t="s">
+      <c r="AS1" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="S1" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="T1" s="19" t="s">
+      <c r="AT1" s="28" t="s">
+        <v>44</v>
+      </c>
+      <c r="AU1" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="AV1" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="AW1" s="0"/>
+    </row>
+    <row r="2" s="30" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="30" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="31" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="E2" s="30" t="s">
+        <v>52</v>
+      </c>
+      <c r="F2" s="30" t="n">
+        <v>526</v>
+      </c>
+      <c r="G2" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="H2" s="30" t="s">
+        <v>54</v>
+      </c>
+      <c r="J2" s="32" t="n">
+        <v>34023</v>
+      </c>
+      <c r="K2" s="30" t="s">
+        <v>55</v>
+      </c>
+      <c r="L2" s="30" t="s">
+        <v>56</v>
+      </c>
+      <c r="M2" s="30" t="s">
+        <v>57</v>
+      </c>
+      <c r="N2" s="30" t="s">
+        <v>58</v>
+      </c>
+      <c r="P2" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q2" s="30" t="s">
+        <v>60</v>
+      </c>
+      <c r="T2" s="30" t="s">
+        <v>58</v>
+      </c>
+      <c r="V2" s="30" t="s">
+        <v>61</v>
+      </c>
+      <c r="W2" s="30" t="s">
+        <v>62</v>
+      </c>
+      <c r="X2" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="Y2" s="30" t="s">
+        <v>64</v>
+      </c>
+      <c r="AB2" s="32" t="n">
+        <v>34023</v>
+      </c>
+      <c r="AC2" s="30" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD2" s="30" t="n">
         <v>15</v>
       </c>
-      <c r="U1" s="19" t="s">
-        <v>44</v>
-      </c>
-      <c r="V1" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="W1" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="X1" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="Y1" s="20" t="s">
-        <v>45</v>
-      </c>
-      <c r="Z1" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="AA1" s="21" t="s">
-        <v>21</v>
-      </c>
-      <c r="AB1" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="AC1" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="AD1" s="22" t="s">
-        <v>24</v>
-      </c>
-      <c r="AE1" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="AF1" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="AG1" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="AH1" s="22" t="s">
-        <v>34</v>
-      </c>
-      <c r="AI1" s="23" t="s">
-        <v>27</v>
-      </c>
-      <c r="AJ1" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="AK1" s="24" t="s">
-        <v>28</v>
-      </c>
-      <c r="AL1" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="AM1" s="23" t="s">
-        <v>30</v>
-      </c>
-      <c r="AN1" s="23" t="s">
-        <v>31</v>
-      </c>
-      <c r="AO1" s="23" t="s">
-        <v>32</v>
-      </c>
-      <c r="AP1" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="AQ1" s="25" t="s">
-        <v>34</v>
-      </c>
-      <c r="AR1" s="25" t="s">
-        <v>35</v>
-      </c>
-      <c r="AS1" s="25" t="s">
-        <v>36</v>
-      </c>
-      <c r="AT1" s="25" t="s">
-        <v>37</v>
-      </c>
-      <c r="AU1" s="25" t="s">
-        <v>38</v>
-      </c>
-      <c r="AV1" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="AW1" s="26" t="s">
-        <v>49</v>
-      </c>
+      <c r="AI2" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="AJ2" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK2" s="33" t="s">
+        <v>68</v>
+      </c>
+      <c r="AW2" s="0"/>
     </row>
-    <row r="2" s="28" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="28" t="s">
-        <v>50</v>
-      </c>
-      <c r="B2" s="29" t="s">
-        <v>51</v>
-      </c>
-      <c r="C2" s="28" t="s">
+    <row r="3" s="30" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="30" t="s">
+        <v>69</v>
+      </c>
+      <c r="B3" s="31" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" s="30" t="s">
+        <v>71</v>
+      </c>
+      <c r="D3" s="30" t="s">
+        <v>72</v>
+      </c>
+      <c r="F3" s="30" t="n">
+        <v>322</v>
+      </c>
+      <c r="G3" s="30" t="s">
+        <v>73</v>
+      </c>
+      <c r="H3" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="N3" s="30" t="s">
+        <v>75</v>
+      </c>
+      <c r="P3" s="30" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q3" s="30" t="s">
+        <v>60</v>
+      </c>
+      <c r="T3" s="30" t="s">
+        <v>75</v>
+      </c>
+      <c r="V3" s="30" t="s">
+        <v>77</v>
+      </c>
+      <c r="W3" s="30" t="s">
+        <v>62</v>
+      </c>
+      <c r="X3" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="Y3" s="30" t="s">
+        <v>78</v>
+      </c>
+      <c r="AB3" s="32" t="n">
+        <v>42993</v>
+      </c>
+      <c r="AC3" s="30" t="s">
+        <v>79</v>
+      </c>
+      <c r="AD3" s="30" t="s">
+        <v>80</v>
+      </c>
+      <c r="AH3" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="AI3" s="30" t="s">
+        <v>82</v>
+      </c>
+      <c r="AK3" s="30" t="s">
+        <v>83</v>
+      </c>
+      <c r="AQ3" s="30" t="s">
+        <v>84</v>
+      </c>
+      <c r="AR3" s="30" t="s">
+        <v>85</v>
+      </c>
+      <c r="AS3" s="30" t="s">
+        <v>86</v>
+      </c>
+      <c r="AW3" s="0"/>
+    </row>
+    <row r="4" s="30" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="30" t="s">
+        <v>69</v>
+      </c>
+      <c r="AH4" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="AQ4" s="30" t="s">
+        <v>84</v>
+      </c>
+      <c r="AR4" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="AS4" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="AW4" s="0"/>
+    </row>
+    <row r="5" s="30" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="30" t="s">
+        <v>69</v>
+      </c>
+      <c r="AH5" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="AQ5" s="30" t="s">
+        <v>84</v>
+      </c>
+      <c r="AR5" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="AS5" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="AW5" s="0"/>
+    </row>
+    <row r="6" s="30" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="30" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="31" t="s">
+        <v>92</v>
+      </c>
+      <c r="C6" s="30" t="s">
+        <v>93</v>
+      </c>
+      <c r="D6" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="E6" s="30" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="28" t="s">
-        <v>53</v>
-      </c>
-      <c r="E2" s="28" t="s">
-        <v>54</v>
-      </c>
-      <c r="F2" s="28" t="n">
-        <v>526</v>
-      </c>
-      <c r="G2" s="28" t="s">
-        <v>55</v>
-      </c>
-      <c r="H2" s="28" t="s">
-        <v>56</v>
-      </c>
-      <c r="J2" s="30" t="n">
-        <v>34023</v>
-      </c>
-      <c r="K2" s="28" t="s">
-        <v>57</v>
-      </c>
-      <c r="L2" s="28" t="s">
-        <v>58</v>
-      </c>
-      <c r="M2" s="28" t="s">
-        <v>59</v>
-      </c>
-      <c r="N2" s="28" t="s">
+      <c r="F6" s="30" t="n">
+        <v>357</v>
+      </c>
+      <c r="G6" s="30" t="s">
+        <v>73</v>
+      </c>
+      <c r="H6" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="J6" s="32" t="n">
+        <v>42605</v>
+      </c>
+      <c r="K6" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="M6" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="N6" s="30" t="s">
+        <v>75</v>
+      </c>
+      <c r="P6" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="Q6" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="P2" s="28" t="s">
-        <v>61</v>
-      </c>
-      <c r="Q2" s="28" t="s">
+      <c r="T6" s="30" t="s">
+        <v>75</v>
+      </c>
+      <c r="V6" s="30" t="s">
+        <v>77</v>
+      </c>
+      <c r="W6" s="30" t="s">
         <v>62</v>
       </c>
-      <c r="T2" s="28" t="s">
-        <v>60</v>
-      </c>
-      <c r="V2" s="28" t="s">
+      <c r="X6" s="30" t="s">
         <v>63</v>
       </c>
-      <c r="W2" s="28" t="s">
-        <v>64</v>
-      </c>
-      <c r="X2" s="28" t="s">
-        <v>65</v>
-      </c>
-      <c r="Y2" s="28" t="s">
-        <v>66</v>
-      </c>
-      <c r="AB2" s="30" t="n">
-        <v>34023</v>
-      </c>
-      <c r="AC2" s="28" t="s">
+      <c r="Y6" s="30" t="s">
+        <v>78</v>
+      </c>
+      <c r="AC6" s="30" t="s">
+        <v>79</v>
+      </c>
+      <c r="AI6" s="30" t="s">
+        <v>98</v>
+      </c>
+      <c r="AJ6" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="AD2" s="28" t="n">
-        <v>15</v>
-      </c>
-      <c r="AI2" s="28" t="s">
-        <v>68</v>
-      </c>
-      <c r="AJ2" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="AK2" s="31" t="s">
-        <v>70</v>
-      </c>
+      <c r="AW6" s="0"/>
     </row>
-    <row r="3" s="28" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="B3" s="29" t="s">
-        <v>72</v>
-      </c>
-      <c r="C3" s="28" t="s">
-        <v>73</v>
-      </c>
-      <c r="D3" s="28" t="s">
-        <v>74</v>
-      </c>
-      <c r="F3" s="28" t="n">
-        <v>322</v>
-      </c>
-      <c r="G3" s="28" t="s">
+    <row r="7" s="30" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="30" t="s">
+        <v>91</v>
+      </c>
+      <c r="N7" s="30" t="s">
+        <v>62</v>
+      </c>
+      <c r="P7" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="T7" s="30" t="s">
         <v>75</v>
       </c>
-      <c r="H3" s="28" t="s">
-        <v>76</v>
-      </c>
-      <c r="N3" s="28" t="s">
+      <c r="V7" s="30" t="s">
         <v>77</v>
       </c>
-      <c r="P3" s="28" t="s">
+      <c r="W7" s="30" t="s">
+        <v>62</v>
+      </c>
+      <c r="X7" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="Y7" s="30" t="s">
         <v>78</v>
       </c>
-      <c r="Q3" s="28" t="s">
-        <v>62</v>
-      </c>
-      <c r="T3" s="28" t="s">
-        <v>77</v>
-      </c>
-      <c r="V3" s="28" t="s">
-        <v>79</v>
-      </c>
-      <c r="W3" s="28" t="s">
-        <v>64</v>
-      </c>
-      <c r="X3" s="28" t="s">
-        <v>65</v>
-      </c>
-      <c r="Y3" s="28" t="s">
-        <v>80</v>
-      </c>
-      <c r="AB3" s="30" t="n">
-        <v>42993</v>
-      </c>
-      <c r="AC3" s="28" t="s">
-        <v>81</v>
-      </c>
-      <c r="AD3" s="28" t="s">
-        <v>82</v>
-      </c>
-      <c r="AH3" s="28" t="s">
-        <v>83</v>
-      </c>
-      <c r="AI3" s="28" t="s">
-        <v>84</v>
-      </c>
-      <c r="AK3" s="28" t="s">
-        <v>85</v>
-      </c>
-      <c r="AQ3" s="28" t="s">
-        <v>83</v>
-      </c>
-      <c r="AR3" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="AS3" s="28" t="s">
-        <v>87</v>
-      </c>
-      <c r="AT3" s="28" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="4" s="28" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="AH4" s="28" t="s">
-        <v>83</v>
-      </c>
-      <c r="AQ4" s="28" t="s">
-        <v>83</v>
-      </c>
-      <c r="AR4" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="AS4" s="28" t="s">
-        <v>89</v>
-      </c>
-      <c r="AT4" s="28" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="5" s="28" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="AH5" s="28" t="s">
-        <v>83</v>
-      </c>
-      <c r="AQ5" s="28" t="s">
-        <v>83</v>
-      </c>
-      <c r="AR5" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="AS5" s="28" t="s">
-        <v>91</v>
-      </c>
-      <c r="AT5" s="28" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="6" s="28" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="B6" s="29" t="s">
-        <v>94</v>
-      </c>
-      <c r="C6" s="28" t="s">
-        <v>95</v>
-      </c>
-      <c r="D6" s="28" t="s">
-        <v>96</v>
-      </c>
-      <c r="E6" s="28" t="s">
-        <v>54</v>
-      </c>
-      <c r="F6" s="28" t="n">
-        <v>357</v>
-      </c>
-      <c r="G6" s="28" t="s">
-        <v>75</v>
-      </c>
-      <c r="H6" s="28" t="s">
-        <v>76</v>
-      </c>
-      <c r="J6" s="30" t="n">
-        <v>42605</v>
-      </c>
-      <c r="K6" s="28" t="s">
-        <v>97</v>
-      </c>
-      <c r="M6" s="28" t="s">
-        <v>98</v>
-      </c>
-      <c r="N6" s="28" t="s">
-        <v>77</v>
-      </c>
-      <c r="P6" s="28" t="s">
+      <c r="AC7" s="30" t="s">
         <v>99</v>
       </c>
-      <c r="Q6" s="28" t="s">
-        <v>62</v>
-      </c>
-      <c r="T6" s="28" t="s">
-        <v>77</v>
-      </c>
-      <c r="V6" s="28" t="s">
-        <v>79</v>
-      </c>
-      <c r="W6" s="28" t="s">
-        <v>64</v>
-      </c>
-      <c r="X6" s="28" t="s">
-        <v>65</v>
-      </c>
-      <c r="Y6" s="28" t="s">
-        <v>80</v>
-      </c>
-      <c r="AC6" s="28" t="s">
-        <v>81</v>
-      </c>
-      <c r="AI6" s="28" t="s">
+      <c r="AI7" s="30" t="s">
         <v>100</v>
       </c>
-      <c r="AJ6" s="28" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="7" s="28" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="N7" s="28" t="s">
-        <v>64</v>
-      </c>
-      <c r="P7" s="28" t="s">
-        <v>99</v>
-      </c>
-      <c r="T7" s="28" t="s">
-        <v>77</v>
-      </c>
-      <c r="V7" s="28" t="s">
-        <v>79</v>
-      </c>
-      <c r="W7" s="28" t="s">
-        <v>64</v>
-      </c>
-      <c r="X7" s="28" t="s">
-        <v>65</v>
-      </c>
-      <c r="Y7" s="28" t="s">
-        <v>80</v>
-      </c>
-      <c r="AC7" s="28" t="s">
+      <c r="AK7" s="30" t="s">
         <v>101</v>
       </c>
-      <c r="AI7" s="28" t="s">
-        <v>102</v>
-      </c>
-      <c r="AK7" s="28" t="s">
-        <v>103</v>
-      </c>
+      <c r="AW7" s="0"/>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B8" s="31" t="s">
+        <v>103</v>
+      </c>
+      <c r="C8" s="33" t="s">
         <v>104</v>
       </c>
-      <c r="B8" s="29" t="s">
+      <c r="D8" s="33" t="s">
         <v>105</v>
       </c>
-      <c r="C8" s="31" t="s">
-        <v>106</v>
-      </c>
-      <c r="D8" s="31" t="s">
-        <v>107</v>
-      </c>
       <c r="E8" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F8" s="1" t="n">
         <v>582</v>
       </c>
       <c r="G8" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="J8" s="34" t="n">
+        <v>38520</v>
+      </c>
+      <c r="K8" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="L8" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="J8" s="32" t="n">
-        <v>38520</v>
-      </c>
-      <c r="K8" s="1" t="s">
+      <c r="M8" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="N8" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="L8" s="1" t="s">
+      <c r="P8" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="M8" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="N8" s="1" t="s">
+      <c r="Q8" s="1" t="s">
         <v>112</v>
-      </c>
-      <c r="P8" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="Q8" s="1" t="s">
-        <v>114</v>
       </c>
       <c r="R8" s="1"/>
       <c r="T8" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="V8" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="W8" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="X8" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="Y8" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="V8" s="1" t="s">
+      <c r="Z8" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="AB8" s="34" t="s">
+        <v>117</v>
+      </c>
+      <c r="AC8" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="W8" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="X8" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="Y8" s="0" t="s">
-        <v>117</v>
-      </c>
-      <c r="Z8" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="AB8" s="32" t="s">
-        <v>119</v>
-      </c>
-      <c r="AC8" s="1" t="s">
-        <v>81</v>
       </c>
       <c r="AD8" s="1" t="n">
         <v>3</v>
       </c>
       <c r="AI8" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="AJ8" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B9" s="35" t="s">
+        <v>120</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B9" s="33" t="s">
+      <c r="D9" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>124</v>
-      </c>
       <c r="E9" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F9" s="1" t="n">
         <v>651</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="H9" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="J9" s="34" t="n">
+        <v>30706</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="M9" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="J9" s="32" t="n">
-        <v>30706</v>
-      </c>
-      <c r="K9" s="1" t="s">
+      <c r="N9" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="M9" s="1" t="s">
+      <c r="P9" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="N9" s="1" t="s">
+      <c r="Q9" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="P9" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="Q9" s="1" t="s">
-        <v>130</v>
       </c>
       <c r="R9" s="1"/>
       <c r="T9" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="U9" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="V9" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="W9" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="X9" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="Y9" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="AB9" s="34" t="n">
+        <v>30706</v>
+      </c>
+      <c r="AC9" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="U9" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="V9" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="W9" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="X9" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="Y9" s="0" t="s">
-        <v>132</v>
-      </c>
-      <c r="AB9" s="32" t="n">
-        <v>30706</v>
-      </c>
-      <c r="AC9" s="1" t="s">
-        <v>133</v>
       </c>
       <c r="AD9" s="1" t="n">
         <v>8</v>
       </c>
       <c r="AE9" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="AI9" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="AL9" s="1" t="s">
         <v>134</v>
-      </c>
-      <c r="AI9" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="AL9" s="1" t="s">
-        <v>136</v>
       </c>
       <c r="AM9" s="1" t="n">
         <v>2003</v>
       </c>
-      <c r="AN9" s="34" t="s">
-        <v>137</v>
-      </c>
-      <c r="AP9" s="35" t="s">
-        <v>138</v>
+      <c r="AN9" s="36" t="s">
+        <v>135</v>
+      </c>
+      <c r="AP9" s="37" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1"/>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="P10" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="Q10" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="P10" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="Q10" s="1" t="s">
-        <v>145</v>
       </c>
       <c r="R10" s="1"/>
       <c r="T10" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="V10" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="W10" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="V10" s="1" t="s">
+      <c r="X10" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="W10" s="1" t="s">
+      <c r="AI10" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="X10" s="1" t="s">
+      <c r="AL10" s="1" t="s">
         <v>149</v>
-      </c>
-      <c r="AI10" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="AL10" s="1" t="s">
-        <v>151</v>
       </c>
       <c r="AM10" s="1" t="n">
         <v>2005</v>
       </c>
       <c r="AN10" s="1" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="G11" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="N11" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="P11" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="T11" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="G11" s="1" t="s">
+      <c r="U11" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="V11" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="W11" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="X11" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="Y11" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="N11" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="P11" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="T11" s="1" t="s">
+      <c r="AI11" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="U11" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="V11" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="W11" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="X11" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="Y11" s="1" t="s">
+      <c r="AL11" s="1" t="s">
         <v>158</v>
-      </c>
-      <c r="AI11" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="AL11" s="1" t="s">
-        <v>160</v>
       </c>
       <c r="AM11" s="1" t="n">
         <v>1965</v>
       </c>
       <c r="AP11" s="1" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="G12" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="P12" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="T12" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="G12" s="1" t="s">
+      <c r="V12" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="P12" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="T12" s="1" t="s">
+      <c r="W12" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="AA12" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="V12" s="1" t="s">
+      <c r="AK12" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="W12" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="AA12" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="AK12" s="1" t="s">
-        <v>168</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add verbatim identification field to dataset template
</commit_message>
<xml_diff>
--- a/template/public/template.xlsx
+++ b/template/public/template.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="168">
   <si>
     <t xml:space="preserve">site_code</t>
   </si>
@@ -105,6 +105,9 @@
   </si>
   <si>
     <t xml:space="preserve">identified_by</t>
+  </si>
+  <si>
+    <t xml:space="preserve">verbatim_identification</t>
   </si>
   <si>
     <t xml:space="preserve">specimen_quantity</t>
@@ -941,7 +944,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:BA1"/>
+  <dimension ref="A1:BB1"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="11.53"/>
@@ -958,18 +961,23 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="13.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="20" style="1" width="13.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="23" style="1" width="14.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="14.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="1" width="17.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="1" width="14.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="20.16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="27" style="1" width="16.69"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="1" width="18.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="1" width="19.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="1" width="33.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="33" style="1" width="16.69"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="35" style="1" width="20.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="40" style="1" width="13.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="43" style="1" width="26.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="1" width="20.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="46" min="46" style="1" width="19.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="27" style="1" width="16.69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="1" width="18.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="1" width="16.69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="1" width="18.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="1" width="19.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="1" width="33.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="34" style="1" width="16.69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="36" style="1" width="20.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="42" min="41" style="1" width="13.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="1" width="26.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="1" width="20.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="47" min="47" style="1" width="19.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="48" min="48" style="0" width="18.88"/>
   </cols>
   <sheetData>
     <row r="1" s="16" customFormat="true" ht="29.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1057,7 +1065,7 @@
       <c r="AB1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="10" t="s">
+      <c r="AC1" s="9" t="s">
         <v>28</v>
       </c>
       <c r="AD1" s="10" t="s">
@@ -1072,16 +1080,16 @@
       <c r="AG1" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="11" t="s">
+      <c r="AH1" s="10" t="s">
         <v>33</v>
       </c>
       <c r="AI1" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" s="12" t="s">
+      <c r="AJ1" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" s="11" t="s">
+      <c r="AK1" s="12" t="s">
         <v>36</v>
       </c>
       <c r="AL1" s="11" t="s">
@@ -1096,30 +1104,33 @@
       <c r="AO1" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" s="13" t="s">
+      <c r="AP1" s="11" t="s">
         <v>41</v>
       </c>
       <c r="AQ1" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" s="14" t="s">
+      <c r="AR1" s="13" t="s">
         <v>43</v>
       </c>
       <c r="AS1" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="AT1" s="15" t="s">
+      <c r="AT1" s="14" t="s">
         <v>45</v>
       </c>
       <c r="AU1" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="AV1" s="1"/>
+      <c r="AV1" s="15" t="s">
+        <v>47</v>
+      </c>
       <c r="AW1" s="1"/>
       <c r="AX1" s="1"/>
       <c r="AY1" s="1"/>
       <c r="AZ1" s="1"/>
-      <c r="BA1" s="0"/>
+      <c r="BA1" s="1"/>
+      <c r="BB1" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1156,7 +1167,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="1" width="34.49"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="47" min="47" style="1" width="19.27"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="48" min="48" style="1" width="16.96"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" s="29" customFormat="true" ht="29.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1203,7 +1214,7 @@
         <v>13</v>
       </c>
       <c r="O1" s="21" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="P1" s="20" t="s">
         <v>14</v>
@@ -1248,667 +1259,667 @@
         <v>27</v>
       </c>
       <c r="AD1" s="25" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="AE1" s="25" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="AF1" s="25" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="AG1" s="25" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="AH1" s="25" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="AI1" s="26" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="AJ1" s="26" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="AK1" s="27" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="AL1" s="26" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="AM1" s="26" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="AN1" s="26" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="AO1" s="26" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="AP1" s="26" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="AQ1" s="28" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="AR1" s="28" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="AS1" s="28" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="AT1" s="28" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AU1" s="15" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AV1" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="AW1" s="0"/>
+        <v>47</v>
+      </c>
+      <c r="AW1" s="1"/>
     </row>
     <row r="2" s="30" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="30" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B2" s="31" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C2" s="30" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D2" s="30" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E2" s="30" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F2" s="30" t="n">
         <v>526</v>
       </c>
       <c r="G2" s="30" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H2" s="30" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J2" s="32" t="n">
         <v>34023</v>
       </c>
       <c r="K2" s="30" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L2" s="30" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="M2" s="30" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N2" s="30" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="P2" s="30" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q2" s="30" t="s">
+        <v>61</v>
+      </c>
+      <c r="T2" s="30" t="s">
         <v>59</v>
       </c>
-      <c r="Q2" s="30" t="s">
-        <v>60</v>
-      </c>
-      <c r="T2" s="30" t="s">
-        <v>58</v>
-      </c>
       <c r="V2" s="30" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="W2" s="30" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="X2" s="30" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Y2" s="30" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AB2" s="32" t="n">
         <v>34023</v>
       </c>
       <c r="AC2" s="30" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="AD2" s="30" t="n">
         <v>15</v>
       </c>
       <c r="AI2" s="30" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="AJ2" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="AK2" s="33" t="s">
-        <v>68</v>
-      </c>
-      <c r="AW2" s="0"/>
+        <v>69</v>
+      </c>
+      <c r="AW2" s="1"/>
     </row>
     <row r="3" s="30" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="30" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C3" s="30" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D3" s="30" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F3" s="30" t="n">
         <v>322</v>
       </c>
       <c r="G3" s="30" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H3" s="30" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="N3" s="30" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="P3" s="30" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q3" s="30" t="s">
+        <v>61</v>
+      </c>
+      <c r="T3" s="30" t="s">
         <v>76</v>
       </c>
-      <c r="Q3" s="30" t="s">
-        <v>60</v>
-      </c>
-      <c r="T3" s="30" t="s">
-        <v>75</v>
-      </c>
       <c r="V3" s="30" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="W3" s="30" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="X3" s="30" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Y3" s="30" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="AB3" s="32" t="n">
         <v>42993</v>
       </c>
       <c r="AC3" s="30" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="AD3" s="30" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="AH3" s="30" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="AI3" s="30" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="AK3" s="30" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="AQ3" s="30" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="AR3" s="30" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AS3" s="30" t="s">
-        <v>86</v>
-      </c>
-      <c r="AW3" s="0"/>
+        <v>87</v>
+      </c>
+      <c r="AW3" s="1"/>
     </row>
     <row r="4" s="30" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="30" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="AH4" s="30" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="AQ4" s="30" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="AR4" s="30" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="AS4" s="30" t="s">
-        <v>88</v>
-      </c>
-      <c r="AW4" s="0"/>
+        <v>89</v>
+      </c>
+      <c r="AW4" s="1"/>
     </row>
     <row r="5" s="30" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="30" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="AH5" s="30" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="AQ5" s="30" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="AR5" s="30" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="AS5" s="30" t="s">
-        <v>90</v>
-      </c>
-      <c r="AW5" s="0"/>
+        <v>91</v>
+      </c>
+      <c r="AW5" s="1"/>
     </row>
     <row r="6" s="30" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="30" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B6" s="31" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C6" s="30" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D6" s="30" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E6" s="30" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F6" s="30" t="n">
         <v>357</v>
       </c>
       <c r="G6" s="30" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H6" s="30" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J6" s="32" t="n">
         <v>42605</v>
       </c>
       <c r="K6" s="30" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="M6" s="30" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="N6" s="30" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="P6" s="30" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="Q6" s="30" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="T6" s="30" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="V6" s="30" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="W6" s="30" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="X6" s="30" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Y6" s="30" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="AC6" s="30" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="AI6" s="30" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AJ6" s="30" t="s">
-        <v>67</v>
-      </c>
-      <c r="AW6" s="0"/>
+        <v>68</v>
+      </c>
+      <c r="AW6" s="1"/>
     </row>
     <row r="7" s="30" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="30" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N7" s="30" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="P7" s="30" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="T7" s="30" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="V7" s="30" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="W7" s="30" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="X7" s="30" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Y7" s="30" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="AC7" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AI7" s="30" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="AK7" s="30" t="s">
-        <v>101</v>
-      </c>
-      <c r="AW7" s="0"/>
+        <v>102</v>
+      </c>
+      <c r="AW7" s="1"/>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B8" s="31" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F8" s="1" t="n">
         <v>582</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J8" s="34" t="n">
         <v>38520</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="R8" s="1"/>
       <c r="T8" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="W8" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="X8" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Y8" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Z8" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AB8" s="34" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AC8" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="AD8" s="1" t="n">
         <v>3</v>
       </c>
       <c r="AI8" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AJ8" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B9" s="35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F9" s="1" t="n">
         <v>651</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J9" s="34" t="n">
         <v>30706</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="R9" s="1"/>
       <c r="T9" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="V9" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="W9" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="X9" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Y9" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AB9" s="34" t="n">
         <v>30706</v>
       </c>
       <c r="AC9" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AD9" s="1" t="n">
         <v>8</v>
       </c>
       <c r="AE9" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="AI9" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="AL9" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="AM9" s="1" t="n">
         <v>2003</v>
       </c>
       <c r="AN9" s="36" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AP9" s="37" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1"/>
       <c r="B10" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="R10" s="1"/>
       <c r="T10" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="V10" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="W10" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="X10" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AI10" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="AL10" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="AM10" s="1" t="n">
         <v>2005</v>
       </c>
       <c r="AN10" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="P11" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="T11" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="U11" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="V11" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="W11" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="X11" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Y11" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="AI11" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="AL11" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="AM11" s="1" t="n">
         <v>1965</v>
       </c>
       <c r="AP11" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="T12" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="V12" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="W12" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="AA12" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="AK12" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>